<commit_message>
docs: added daily tracker spreadsheet
</commit_message>
<xml_diff>
--- a/backend/Backend-Daily-Tracker.xlsx
+++ b/backend/Backend-Daily-Tracker.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="90">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -478,6 +478,12 @@
   </si>
   <si>
     <t>Tested the new system after the whole update for security flaws, logged in account issues. Found that reviews were not linked to the businesses yet</t>
+  </si>
+  <si>
+    <t>Fixed the stale admin session issue on page load and added role-based login redirects, so admins and regular users land on the correct pages after signing in. Updated the admin navbar and logout so logging out now takes the user to the login page. Improved admin session security by making sessions end when the browser closes and shortening the admin token lifetime to 8 hours. Added a script to import WordPress reviews into the platform. Updated the zustand dependency to version 4.5.7 and refreshed the generated Next.js type file. Investigated why the admin-managed hero images were not appearing on the homepage. The cause was server-side caching combined with a missing browser refetch, and I fixed it so the homepage now shows the latest hero images. Also fixed the disabled "Email announcement" button on the Customers page, which stayed greyed out for owners with a single business. Finalized the project structure and updated .gitignore so that environment files, uploads, and private user data are not pushed to GitHub.</t>
+  </si>
+  <si>
+    <t>1. Fix stale admin session on load; role-based login redirect; admin navbar and logout to /login           2. Admin sessions end when the browser closes; 8h admin token                 3. Add WordPress review import script Bump zustand to 4.5.7 and update generated next-env.d.ts                           5. Fix hero images not refreshing and enable email announcement for single-business owners      6. fix: finalized project changes and hidden private datas                     7. docs: added daily tracker spreadsheet</t>
   </si>
 </sst>
 </file>
@@ -1997,18 +2003,26 @@
       </c>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="277.2" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>34</v>
       </c>
-      <c r="B38" s="3"/>
+      <c r="B38" s="5">
+        <v>46301</v>
+      </c>
       <c r="C38" s="2"/>
-      <c r="D38" s="3"/>
+      <c r="D38" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="E38" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F38" s="2"/>
-      <c r="G38" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="H38" s="3"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>